<commit_message>
list trunk-group changed to display hardcoded values from the csv file. Status trunk yet to be changed
</commit_message>
<xml_diff>
--- a/backend/latest_avaya_page_log.xlsx
+++ b/backend/latest_avaya_page_log.xlsx
@@ -454,7 +454,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:07</t>
+          <t>2025-12-03 19:36:23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -485,7 +485,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:07</t>
+          <t>2025-12-03 19:36:23</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -495,7 +495,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mon Nov 24 12:24:07 IST 2025</t>
+          <t>Wed Dec  3 19:36:23 IST 2025</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -503,7 +503,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:07</t>
+          <t>2025-12-03 19:36:24</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -513,7 +513,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>12:24:07 up 3 days, 4 min,  1 user,  load average: 0.02, 0.04, 0.05</t>
+          <t>19:36:24 up 12 days,  7:16,  1 user,  load average: 0.06, 0.05, 0.05</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -521,7 +521,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:08</t>
+          <t>2025-12-03 19:36:24</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -537,7 +537,7 @@
 tmpfs           1.7G     0  1.7G   0% /dev/shm
 tmpfs           1.7G  8.9M  1.6G   1% /run
 tmpfs           1.7G     0  1.7G   0% /sys/fs/cgroup
-/dev/sdb5        35G  899M   35G   3% /var
+/dev/sdb5        35G  901M   35G   3% /var
 /dev/sdb2       5.0G   33M  5.0G   1% /var/log/audit
 /dev/sdb1       5.0G   33M  5.0G   1% /var/home
 /dev/sdb3       5.0G   33M  5.0G   1% /var/tmp
@@ -550,7 +550,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:09</t>
+          <t>2025-12-03 19:36:25</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -566,7 +566,7 @@
 tmpfs            1682316       0   1682316   0% /dev/shm
 tmpfs            1682316    9044   1673272   1% /run
 tmpfs            1682316       0   1682316   0% /sys/fs/cgroup
-/dev/sdb5       36680196  920024  35760172   3% /var
+/dev/sdb5       36680196  921904  35758292   3% /var
 /dev/sdb2        5232640   32992   5199648   1% /var/log/audit
 /dev/sdb1        5232640   33212   5199428   1% /var/home
 /dev/sdb3        5232640   33112   5199528   1% /var/tmp
@@ -579,7 +579,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:09</t>
+          <t>2025-12-03 19:36:25</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -599,7 +599,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:10</t>
+          <t>2025-12-03 19:36:26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -622,7 +622,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:10</t>
+          <t>2025-12-03 19:36:26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -649,7 +649,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:11</t>
+          <t>2025-12-03 19:36:27</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -711,7 +711,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:33</t>
+          <t>2025-12-03 19:36:49</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -728,7 +728,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:33</t>
+          <t>2025-12-03 19:36:49</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -745,7 +745,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:33</t>
+          <t>2025-12-03 19:36:49</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -762,7 +762,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:33</t>
+          <t>2025-12-03 19:36:49</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -778,7 +778,7 @@
  Link           Busy  Server           State         Sent     Rcvd
 -1 10no aes7038        established 15     15     
+1 10no aes7038        established 14     14     
  7                                                                                Command successfully completed87                8Command:</t>
         </is>
@@ -787,7 +787,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:33</t>
+          <t>2025-12-03 19:36:49</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -804,7 +804,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:33</t>
+          <t>2025-12-03 19:36:49</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -821,7 +821,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:33</t>
+          <t>2025-12-03 19:36:49</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>list measurements outage-trunk last-hour                                                                                7                                                                                87list measurements outage-trunk last-hour 8                                                                                7       Page   18Switch Name:                     Date: 12:24 pm  MON NOV 24, 2025 
+          <t>list measurements outage-trunk last-hour                                                                                7                                                                                87list measurements outage-trunk last-hour 8                                                                                7       Page   18Switch Name:                     Date: 7:36 pm  WED DEC 3, 2025   
  TRUNK OUT OF SERVICE REPORT
 @@ -841,31 +841,31 @@
  No.   Type  Dir  Size  Mbr#   Outages
 +1   sip two10  1   1   
++1   sip two10  2   1   
++1   sip two10  3   1   
++1   sip two10  4   1   
++1   sip two10  5   1   
++1   sip two10  6   1   
++1   sip two10  7   1   
++1   sip two10  8   1   
++1   sip two10  9   1   
++1   sip two10  10  1   
+ 4   sip two50  1   1   
  4   sip two50  2   1   
  4   sip two50  3   1   
--4   sip two50  4   1   
--4   sip two50  5   1   
--4   sip two50  6   1   
--4   sip two50  7   1   
--4   sip two50  8   1   
--4   sip two50  9   1   
--4   sip two50  10  1   
--4   sip two50  11  1   
--4   sip two50  12  1   
--4   sip two50  13  1   
  7                                                                                		press CANCEL to quit --  press NEXT PAGE to continue8</t>
         </is>
@@ -874,7 +874,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:33</t>
+          <t>2025-12-03 19:36:49</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -891,7 +891,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:33</t>
+          <t>2025-12-03 19:36:49</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -908,7 +908,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-11-24 12:24:33</t>
+          <t>2025-12-03 19:36:49</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">

</xml_diff>